<commit_message>
add new data 0429
</commit_message>
<xml_diff>
--- a/data/Hermenches/cost/cost_report.xlsx
+++ b/data/Hermenches/cost/cost_report.xlsx
@@ -482,30 +482,30 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>87.7346164127494</v>
+        <v>87.37694928176012</v>
       </c>
       <c r="C2" t="n">
-        <v>1919.939378820379</v>
+        <v>3628.587227396264</v>
       </c>
       <c r="D2" t="n">
-        <v>902.0201422778952</v>
+        <v>-4023.156897879823</v>
       </c>
       <c r="E2" t="n">
-        <v>916.8171533422656</v>
+        <v>1924.485480556701</v>
       </c>
       <c r="F2" t="n">
-        <v>8012.848064172324</v>
+        <v>9359.994047064463</v>
       </c>
       <c r="G2" t="n">
-        <v>11839.35935502562</v>
+        <v>10977.28680641937</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>all</t>
+          <t>base</t>
         </is>
       </c>
       <c r="I2" t="n">
-        <v>0.148982215081841</v>
+        <v>0.1381342059961053</v>
       </c>
     </row>
     <row r="3">
@@ -518,27 +518,27 @@
         <v>87.37694928176012</v>
       </c>
       <c r="C3" t="n">
-        <v>3628.587227396264</v>
+        <v>3626.002848516887</v>
       </c>
       <c r="D3" t="n">
-        <v>-4023.156897879823</v>
+        <v>-3870.026066165092</v>
       </c>
       <c r="E3" t="n">
-        <v>1924.485480556701</v>
+        <v>2100.831012913118</v>
       </c>
       <c r="F3" t="n">
-        <v>9359.994047064463</v>
+        <v>9741.00457562948</v>
       </c>
       <c r="G3" t="n">
-        <v>10977.28680641937</v>
+        <v>11685.18932017615</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>base</t>
+          <t>cp_dr</t>
         </is>
       </c>
       <c r="I3" t="n">
-        <v>0.1381342059961053</v>
+        <v>0.147042195136305</v>
       </c>
     </row>
     <row r="4">
@@ -548,30 +548,30 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>87.37694928176012</v>
+        <v>87.7346164127494</v>
       </c>
       <c r="C4" t="n">
-        <v>3626.002848516887</v>
+        <v>1919.939378820379</v>
       </c>
       <c r="D4" t="n">
-        <v>-3870.026066165092</v>
+        <v>902.0201422778952</v>
       </c>
       <c r="E4" t="n">
-        <v>2100.831012913118</v>
+        <v>916.8171533422656</v>
       </c>
       <c r="F4" t="n">
-        <v>9741.00457562948</v>
+        <v>8012.848064172324</v>
       </c>
       <c r="G4" t="n">
-        <v>11685.18932017615</v>
+        <v>11839.35935502562</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>cp_dr</t>
+          <t>all</t>
         </is>
       </c>
       <c r="I4" t="n">
-        <v>0.147042195136305</v>
+        <v>0.148982215081841</v>
       </c>
     </row>
     <row r="5">

</xml_diff>